<commit_message>
Completed member 2 intent classification module
</commit_message>
<xml_diff>
--- a/cleaned_dataset.xlsx
+++ b/cleaned_dataset.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,28 +425,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D369"/>
+  <dimension ref="A1:E369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tulu_text</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>english</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>intent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>merged_intent</t>
         </is>
       </c>
     </row>
@@ -459,6 +476,11 @@
           <t>greeting</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>greeting</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,6 +503,11 @@
           <t>identity</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -503,6 +530,11 @@
           <t>daily_activity</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -525,6 +557,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -547,6 +584,11 @@
           <t>future_action</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>future_action</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -569,6 +611,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -591,6 +638,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -613,6 +665,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -635,6 +692,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -657,6 +719,11 @@
           <t>request_help</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>help</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -679,6 +746,11 @@
           <t>identity</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -701,6 +773,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -723,6 +800,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -745,6 +827,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -767,6 +854,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -789,6 +881,11 @@
           <t>daily_activity</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -811,6 +908,11 @@
           <t>daily_activity</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -833,6 +935,11 @@
           <t>daily_activity</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -855,6 +962,11 @@
           <t>daily_activity</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -877,6 +989,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -899,6 +1016,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -921,6 +1043,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -943,6 +1070,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -965,6 +1097,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -987,6 +1124,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1009,6 +1151,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1031,6 +1178,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1053,6 +1205,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1075,6 +1232,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1097,6 +1259,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1119,6 +1286,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1141,6 +1313,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1163,6 +1340,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1185,6 +1367,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1207,6 +1394,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1229,6 +1421,11 @@
           <t>opinion</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>opinion</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1251,6 +1448,11 @@
           <t>opinion</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>opinion</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1273,6 +1475,11 @@
           <t>opinion</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>opinion</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1295,6 +1502,11 @@
           <t>opinion</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>opinion</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1317,6 +1529,11 @@
           <t>opinion</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>opinion</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1339,6 +1556,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1361,6 +1583,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1383,6 +1610,11 @@
           <t>appreciation</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>appreciation</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1405,6 +1637,11 @@
           <t>appreciation</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>appreciation</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1427,6 +1664,11 @@
           <t>appreciation</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>appreciation</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1449,6 +1691,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1471,6 +1718,11 @@
           <t>future_action</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>future_action</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1493,6 +1745,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1515,6 +1772,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1537,6 +1799,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1559,6 +1826,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1581,6 +1853,11 @@
           <t>opinion</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>opinion</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1603,6 +1880,11 @@
           <t>opinion</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>opinion</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1625,6 +1907,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1647,6 +1934,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1669,6 +1961,11 @@
           <t>emotion</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1691,6 +1988,11 @@
           <t>emotion</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1713,6 +2015,11 @@
           <t>emotion</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1735,6 +2042,11 @@
           <t>emotion</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1757,6 +2069,11 @@
           <t>emotion</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1779,6 +2096,11 @@
           <t>information_request</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1801,6 +2123,11 @@
           <t>information_request</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1823,6 +2150,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1845,6 +2177,11 @@
           <t>personal_status</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1867,6 +2204,11 @@
           <t>question_general</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>information_request</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1889,6 +2231,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1911,6 +2258,11 @@
           <t>instruction</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>instruction</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1933,6 +2285,11 @@
           <t>future_action</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>future_action</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1955,6 +2312,11 @@
           <t>future_action</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>future_action</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1977,6 +2339,11 @@
           <t>polite_expression</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>polite_expression</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1999,6 +2366,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2021,6 +2393,11 @@
           <t>temperature</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2043,6 +2420,11 @@
           <t>rain</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2065,6 +2447,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2087,6 +2474,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2109,6 +2501,11 @@
           <t>forecast</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2131,6 +2528,11 @@
           <t>forecast</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2153,6 +2555,11 @@
           <t>rain</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2175,6 +2582,11 @@
           <t>temperature</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2197,6 +2609,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2219,6 +2636,11 @@
           <t>temperature</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2241,6 +2663,11 @@
           <t>temperature</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2263,6 +2690,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2285,6 +2717,11 @@
           <t>humidity</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2307,6 +2744,11 @@
           <t>rain</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2329,6 +2771,11 @@
           <t>temperature</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2351,6 +2798,11 @@
           <t>wind</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2373,6 +2825,11 @@
           <t>forecast</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2395,6 +2852,11 @@
           <t>forecast</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2417,6 +2879,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2439,6 +2906,11 @@
           <t>temperature</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2461,6 +2933,11 @@
           <t>temperature</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2483,6 +2960,11 @@
           <t>rain</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2505,6 +2987,11 @@
           <t>wind</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2527,6 +3014,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2549,6 +3041,11 @@
           <t>news</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2571,6 +3068,11 @@
           <t>world_news</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2593,6 +3095,11 @@
           <t>headlines</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2615,6 +3122,11 @@
           <t>headlines</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2637,6 +3149,11 @@
           <t>india_news</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2659,6 +3176,11 @@
           <t>breaking_news</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2681,6 +3203,11 @@
           <t>news</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2703,6 +3230,11 @@
           <t>trending_news</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2725,6 +3257,11 @@
           <t>political_news</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2747,6 +3284,11 @@
           <t>political_news</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2769,6 +3311,11 @@
           <t>technology_news</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2791,6 +3338,11 @@
           <t>sports_news</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2813,6 +3365,11 @@
           <t>entertainment_news</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2835,6 +3392,11 @@
           <t>entertainment_news</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2857,6 +3419,11 @@
           <t>local_news</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2879,6 +3446,11 @@
           <t>international_news</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2901,6 +3473,11 @@
           <t>news</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2923,6 +3500,11 @@
           <t>events</t>
         </is>
       </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2945,6 +3527,11 @@
           <t>headlines</t>
         </is>
       </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2967,6 +3554,11 @@
           <t>business_news</t>
         </is>
       </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2989,6 +3581,11 @@
           <t>karnataka_news</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3011,6 +3608,11 @@
           <t>news</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3033,6 +3635,11 @@
           <t>headlines</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3055,6 +3662,11 @@
           <t>top_story</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3077,6 +3689,11 @@
           <t>weather_news</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3099,6 +3716,11 @@
           <t>world_news</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3121,6 +3743,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3143,6 +3770,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3165,6 +3797,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3187,6 +3824,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3209,6 +3851,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3231,6 +3878,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3253,6 +3905,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3275,6 +3932,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3297,6 +3959,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3319,6 +3986,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3341,6 +4013,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3363,6 +4040,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3385,6 +4067,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3407,6 +4094,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3429,6 +4121,11 @@
           <t>day</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3451,6 +4148,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3473,6 +4175,11 @@
           <t>tomorrow_date</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3495,6 +4202,11 @@
           <t>yesterday_date</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3517,6 +4229,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3539,6 +4256,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3561,6 +4283,11 @@
           <t>day</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3583,6 +4310,11 @@
           <t>day_date</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3605,6 +4337,11 @@
           <t>date</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3627,6 +4364,11 @@
           <t>day_date</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3649,6 +4391,11 @@
           <t>date_time</t>
         </is>
       </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3671,6 +4418,11 @@
           <t>year</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3693,6 +4445,11 @@
           <t>month</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3715,6 +4472,11 @@
           <t>eat</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3737,6 +4499,11 @@
           <t>drink</t>
         </is>
       </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3759,6 +4526,11 @@
           <t>bring_item</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3781,6 +4553,11 @@
           <t>cook</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3803,6 +4580,11 @@
           <t>serve_food</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3825,6 +4607,11 @@
           <t>wash</t>
         </is>
       </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3847,6 +4634,11 @@
           <t>clean</t>
         </is>
       </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3869,6 +4661,11 @@
           <t>sweep</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3891,6 +4688,11 @@
           <t>cut</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3913,6 +4715,11 @@
           <t>make_food</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3935,6 +4742,11 @@
           <t>move_come</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3957,6 +4769,11 @@
           <t>move_go</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3979,6 +4796,11 @@
           <t>move_go</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4001,6 +4823,11 @@
           <t>move_walk</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -4023,6 +4850,11 @@
           <t>sit</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -4045,6 +4877,11 @@
           <t>stand</t>
         </is>
       </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -4067,6 +4904,11 @@
           <t>wait</t>
         </is>
       </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4089,6 +4931,11 @@
           <t>move_go</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -4111,6 +4958,11 @@
           <t>move_come</t>
         </is>
       </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -4133,6 +4985,11 @@
           <t>turn</t>
         </is>
       </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -4155,6 +5012,11 @@
           <t>listen</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -4177,6 +5039,11 @@
           <t>speak</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -4199,6 +5066,11 @@
           <t>repeat</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -4221,6 +5093,11 @@
           <t>stop_speak</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -4243,6 +5120,11 @@
           <t>call_person</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -4265,6 +5147,11 @@
           <t>call_person</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4287,6 +5174,11 @@
           <t>ask</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -4309,6 +5201,11 @@
           <t>answer</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -4331,6 +5228,11 @@
           <t>say_truth</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -4353,6 +5255,11 @@
           <t>stop_lie</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -4375,6 +5282,11 @@
           <t>do_work</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -4397,6 +5309,11 @@
           <t>finish_work</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -4419,6 +5336,11 @@
           <t>start_work</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -4441,6 +5363,11 @@
           <t>help</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -4463,6 +5390,11 @@
           <t>lift</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -4485,6 +5417,11 @@
           <t>keep</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -4507,6 +5444,11 @@
           <t>take</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -4529,6 +5471,11 @@
           <t>give</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -4551,6 +5498,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4573,6 +5525,11 @@
           <t>close</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4595,6 +5552,11 @@
           <t>bring_item</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4617,6 +5579,11 @@
           <t>wear</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4639,6 +5606,11 @@
           <t>wash</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4661,6 +5633,11 @@
           <t>dry</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4683,6 +5660,11 @@
           <t>turn_on_light</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>device_control</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4705,6 +5687,11 @@
           <t>turn_off_light</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>device_control</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4727,6 +5714,11 @@
           <t>check</t>
         </is>
       </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4749,6 +5741,11 @@
           <t>look</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -4771,6 +5768,11 @@
           <t>look</t>
         </is>
       </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4793,6 +5795,11 @@
           <t>be_careful</t>
         </is>
       </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4815,6 +5822,11 @@
           <t>move_come</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4837,6 +5849,11 @@
           <t>move_go</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4859,6 +5876,11 @@
           <t>sit</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4881,6 +5903,11 @@
           <t>eat_control</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4903,6 +5930,11 @@
           <t>stop_run</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4925,6 +5957,11 @@
           <t>stay</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4947,6 +5984,11 @@
           <t>follow</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4969,6 +6011,11 @@
           <t>move_go</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4991,6 +6038,11 @@
           <t>wait</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -5013,6 +6065,11 @@
           <t>follow</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -5035,6 +6092,11 @@
           <t>call_person</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -5057,6 +6119,11 @@
           <t>call_person</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -5079,6 +6146,11 @@
           <t>wake_up</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -5101,6 +6173,11 @@
           <t>sleep</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -5123,6 +6200,11 @@
           <t>prepare</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -5145,6 +6227,11 @@
           <t>study</t>
         </is>
       </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -5167,6 +6254,11 @@
           <t>play</t>
         </is>
       </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -5189,6 +6281,11 @@
           <t>move_come</t>
         </is>
       </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -5211,6 +6308,11 @@
           <t>rest</t>
         </is>
       </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -5233,6 +6335,11 @@
           <t>stop_move</t>
         </is>
       </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -5255,6 +6362,11 @@
           <t>bring_item</t>
         </is>
       </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -5277,6 +6389,11 @@
           <t>boil</t>
         </is>
       </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -5299,6 +6416,11 @@
           <t>fill</t>
         </is>
       </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -5321,6 +6443,11 @@
           <t>empty</t>
         </is>
       </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -5343,6 +6470,11 @@
           <t>wash</t>
         </is>
       </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -5365,6 +6497,11 @@
           <t>sweep</t>
         </is>
       </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -5387,6 +6524,11 @@
           <t>dry</t>
         </is>
       </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -5409,6 +6551,11 @@
           <t>fold</t>
         </is>
       </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -5431,6 +6578,11 @@
           <t>wear</t>
         </is>
       </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -5453,6 +6605,11 @@
           <t>remove</t>
         </is>
       </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -5475,6 +6632,11 @@
           <t>tie</t>
         </is>
       </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -5497,6 +6659,11 @@
           <t>untie</t>
         </is>
       </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -5519,6 +6686,11 @@
           <t>turn_on_light</t>
         </is>
       </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>device_control</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -5541,6 +6713,11 @@
           <t>turn_off_light</t>
         </is>
       </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>device_control</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -5563,6 +6740,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -5585,6 +6767,11 @@
           <t>close</t>
         </is>
       </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -5607,6 +6794,11 @@
           <t>lock</t>
         </is>
       </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -5629,6 +6821,11 @@
           <t>unlock</t>
         </is>
       </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -5651,6 +6848,11 @@
           <t>push</t>
         </is>
       </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -5673,6 +6875,11 @@
           <t>pull</t>
         </is>
       </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -5695,6 +6902,11 @@
           <t>carry</t>
         </is>
       </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -5717,6 +6929,11 @@
           <t>keep</t>
         </is>
       </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -5739,6 +6956,11 @@
           <t>bring_item</t>
         </is>
       </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -5761,6 +6983,11 @@
           <t>move_object</t>
         </is>
       </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -5783,6 +7010,11 @@
           <t>arrange</t>
         </is>
       </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -5805,6 +7037,11 @@
           <t>pack</t>
         </is>
       </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -5827,6 +7064,11 @@
           <t>unpack</t>
         </is>
       </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -5849,6 +7091,11 @@
           <t>fix</t>
         </is>
       </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -5871,6 +7118,11 @@
           <t>repair</t>
         </is>
       </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -5893,6 +7145,11 @@
           <t>check</t>
         </is>
       </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -5915,6 +7172,11 @@
           <t>feed_animal</t>
         </is>
       </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -5937,6 +7199,11 @@
           <t>feed_animal</t>
         </is>
       </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -5959,6 +7226,11 @@
           <t>bring_item</t>
         </is>
       </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -5981,6 +7253,11 @@
           <t>clean</t>
         </is>
       </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -6003,6 +7280,11 @@
           <t>tie_animal</t>
         </is>
       </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -6025,6 +7307,11 @@
           <t>untie_animal</t>
         </is>
       </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -6047,6 +7334,11 @@
           <t>take_animal</t>
         </is>
       </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -6069,6 +7361,11 @@
           <t>bring_animal</t>
         </is>
       </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -6091,6 +7388,11 @@
           <t>close</t>
         </is>
       </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -6113,6 +7415,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -6135,6 +7442,11 @@
           <t>move_go</t>
         </is>
       </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -6157,6 +7469,11 @@
           <t>buy</t>
         </is>
       </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -6179,6 +7496,11 @@
           <t>bring_item</t>
         </is>
       </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -6201,6 +7523,11 @@
           <t>take_money</t>
         </is>
       </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -6223,6 +7550,11 @@
           <t>store_money</t>
         </is>
       </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -6245,6 +7577,11 @@
           <t>count_money</t>
         </is>
       </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -6267,6 +7604,11 @@
           <t>give_amount</t>
         </is>
       </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -6289,6 +7631,11 @@
           <t>bring_change</t>
         </is>
       </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -6311,6 +7658,11 @@
           <t>ask_price</t>
         </is>
       </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -6333,6 +7685,11 @@
           <t>pay</t>
         </is>
       </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -6355,6 +7712,11 @@
           <t>wake_up</t>
         </is>
       </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -6377,6 +7739,11 @@
           <t>wake_up</t>
         </is>
       </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -6399,6 +7766,11 @@
           <t>call_person</t>
         </is>
       </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -6421,6 +7793,11 @@
           <t>send</t>
         </is>
       </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -6443,6 +7820,11 @@
           <t>bring_person</t>
         </is>
       </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>bring</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -6465,6 +7847,11 @@
           <t>instruct</t>
         </is>
       </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -6487,6 +7874,11 @@
           <t>instruct</t>
         </is>
       </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -6509,6 +7901,11 @@
           <t>make_sit</t>
         </is>
       </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -6531,6 +7928,11 @@
           <t>allow_go</t>
         </is>
       </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -6553,6 +7955,11 @@
           <t>stop_others</t>
         </is>
       </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -6575,6 +7982,11 @@
           <t>cook</t>
         </is>
       </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -6597,6 +8009,11 @@
           <t>add_ingredient</t>
         </is>
       </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -6619,6 +8036,11 @@
           <t>add_ingredient</t>
         </is>
       </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -6641,6 +8063,11 @@
           <t>stir</t>
         </is>
       </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -6663,6 +8090,11 @@
           <t>taste</t>
         </is>
       </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -6685,6 +8117,11 @@
           <t>serve_food</t>
         </is>
       </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -6707,6 +8144,11 @@
           <t>pour</t>
         </is>
       </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -6729,6 +8171,11 @@
           <t>drink</t>
         </is>
       </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -6751,6 +8198,11 @@
           <t>eat_control</t>
         </is>
       </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -6773,6 +8225,11 @@
           <t>finish_eating</t>
         </is>
       </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -6795,6 +8252,11 @@
           <t>wash_self</t>
         </is>
       </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -6817,6 +8279,11 @@
           <t>comb</t>
         </is>
       </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -6839,6 +8306,11 @@
           <t>wear</t>
         </is>
       </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -6861,6 +8333,11 @@
           <t>remove</t>
         </is>
       </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -6883,6 +8360,11 @@
           <t>sleep</t>
         </is>
       </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -6905,6 +8387,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -6927,6 +8414,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -6949,6 +8441,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -6971,6 +8468,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -6993,6 +8495,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -7015,6 +8522,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -7037,6 +8549,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -7059,6 +8576,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -7081,6 +8603,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -7103,6 +8630,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -7125,6 +8657,11 @@
           <t>placement</t>
         </is>
       </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -7147,6 +8684,11 @@
           <t>movement</t>
         </is>
       </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -7169,6 +8711,11 @@
           <t>silence</t>
         </is>
       </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -7191,6 +8738,11 @@
           <t>device_control</t>
         </is>
       </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>device_control</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -7213,6 +8765,11 @@
           <t>door_control</t>
         </is>
       </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -7235,6 +8792,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -7257,6 +8819,11 @@
           <t>study</t>
         </is>
       </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -7279,6 +8846,11 @@
           <t>positioning</t>
         </is>
       </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>positioning</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -7301,6 +8873,11 @@
           <t>task_execution</t>
         </is>
       </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -7323,6 +8900,11 @@
           <t>communication</t>
         </is>
       </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -7345,6 +8927,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -7367,6 +8954,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -7389,6 +8981,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -7411,6 +9008,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -7433,6 +9035,11 @@
           <t>location</t>
         </is>
       </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -7455,6 +9062,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -7477,6 +9089,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -7499,6 +9116,11 @@
           <t>placement</t>
         </is>
       </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -7521,6 +9143,11 @@
           <t>placement</t>
         </is>
       </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -7543,6 +9170,11 @@
           <t>storytelling</t>
         </is>
       </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -7565,6 +9197,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -7587,6 +9224,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -7609,6 +9251,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -7631,6 +9278,11 @@
           <t>eating</t>
         </is>
       </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -7653,6 +9305,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -7675,6 +9332,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -7697,6 +9359,11 @@
           <t>door_control</t>
         </is>
       </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -7719,6 +9386,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -7741,6 +9413,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -7763,6 +9440,11 @@
           <t>safety</t>
         </is>
       </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -7785,6 +9467,11 @@
           <t>device_activation</t>
         </is>
       </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>device_control</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -7807,6 +9494,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -7829,6 +9521,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -7851,6 +9548,11 @@
           <t>cleaning</t>
         </is>
       </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -7873,6 +9575,11 @@
           <t>preparation</t>
         </is>
       </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -7895,6 +9602,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -7917,6 +9629,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -7939,6 +9656,11 @@
           <t>window_control</t>
         </is>
       </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -7961,6 +9683,11 @@
           <t>weather</t>
         </is>
       </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -7983,6 +9710,11 @@
           <t>location</t>
         </is>
       </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -8005,6 +9737,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -8027,6 +9764,11 @@
           <t>organization</t>
         </is>
       </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -8049,6 +9791,11 @@
           <t>observation</t>
         </is>
       </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -8071,6 +9818,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -8093,6 +9845,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -8115,6 +9872,11 @@
           <t>emotion_expression</t>
         </is>
       </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -8137,6 +9899,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -8159,6 +9926,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -8181,6 +9953,11 @@
           <t xml:space="preserve">placement </t>
         </is>
       </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -8203,6 +9980,11 @@
           <t>attention</t>
         </is>
       </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -8225,6 +10007,11 @@
           <t>time</t>
         </is>
       </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -8247,6 +10034,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -8269,6 +10061,11 @@
           <t>collaboration</t>
         </is>
       </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -8291,6 +10088,11 @@
           <t>study</t>
         </is>
       </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -8313,6 +10115,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -8335,6 +10142,11 @@
           <t>task</t>
         </is>
       </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -8357,6 +10169,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -8379,6 +10196,11 @@
           <t>device_control</t>
         </is>
       </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>device_control</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -8401,6 +10223,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -8423,6 +10250,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -8445,6 +10277,11 @@
           <t>restriction</t>
         </is>
       </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -8467,6 +10304,11 @@
           <t>waiting</t>
         </is>
       </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>wait</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -8489,6 +10331,11 @@
           <t>action</t>
         </is>
       </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -8511,6 +10358,11 @@
           <t>location</t>
         </is>
       </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -8531,6 +10383,11 @@
       <c r="D369" t="inlineStr">
         <is>
           <t>time_awareness</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>safety</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Completed Member 2 intent classification with 80 percent accuracy
</commit_message>
<xml_diff>
--- a/cleaned_dataset.xlsx
+++ b/cleaned_dataset.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,31 +425,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E491"/>
+  <dimension ref="A1:E521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tulu_text</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>english</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>intent</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>merged_intent</t>
         </is>
@@ -13670,6 +13682,816 @@
       <c r="E491" t="inlineStr">
         <is>
           <t xml:space="preserve"> study</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>ಇನಿ ವಾರದ ವಾ ದಿನ</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>What day of the week is today</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>ಇನಿತ ಪೂರ್ತಿ ದಿನಾಂಕ ದಾದ</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>What is today’s full date</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಕೋಡೆ ಒವ್ವು ದಿನ </t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>What day was yesterday</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>tomorrow_day</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>ಎಲ್ಲೆ ದಾದ ದಿನ</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>What day is tomorrow</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>yesterday_day</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಇನಿ ಒವ್ವು ದಿನ </t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>What is the date now</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಈ ತಿಂಗೊಲ್ದ ದಿನಾಂಕ ದಾದ </t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>What is the date this month</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>ಇತ್ತೆ ವಾ ವರ್ಷ</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Which year is now</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>ಒವ್ವು ತಿಂಗೊಲ್ ನಡತೊಂದುಂಡು</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Which month is going on</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>ಇನಿತ  ದಿನ ಬೊಕ್ಕ ದಿನಾಂಕನ್ ಪನ್ಲೆ</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Tell today’s day and date</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>day_date</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>ಇತ್ತೆ ಪೊರ್ತು ಬೊಕ್ಕ ದಿನಾಂಕ ದಾದ</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>What is the time and date now</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>date_time</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>ಗೇಟ್ ತೆರೆಲೆ</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Open the gate</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>open_gate</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>ಗೇಟ್ ನ್ ಮುಚ್ಚುಲೆ</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Close the gate</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>close_gate</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>ಕಿಟಕಿನ್ ತೆರೆಲೆ</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Open the window</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>open_window</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>ಕಿಟಕಿನ್ ಮುಚ್ಚುಲೆ</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Close the window</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>close_window</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>ಬಾಕಿಲ್ ಲಾಕ್ ಮಲ್ಪುಲೆ</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Lock the door</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>lock</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>ಬಾಕಿಲ್ ತೆರೆಯೊಡು</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Unlock the door</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>unlock</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>ಬಾಕಿಲ್ ನ್ ನೂಕುಲೆ</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Push the door</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>push</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>ಬಾಕಿಲ್ ನ್ ಒಯಿಪುಲೆ</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Pull the door</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>pull</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>ಪರದೆನ್ ತೆರೆಲೆ</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Open the curtain</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>open_curtain</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>ಪರದೆನ್ ಮುಚ್ಚುಲೆ</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Close the curtain</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>close_curtain</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>door_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>ಇಲ್ಲ್ ಪೊರ್ಲು ಉಂಡು</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>The house is beautiful</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಈ ಸಾದಿ ಉದ್ದ ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>This road is long</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>ಈ  ಪರ್ನ್ದ್ ಚೀಪೆ ಉಂಡು</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>This fruit is sweet</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಆ ಮರ ಉದ್ದ ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>That tree is tall</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಈ ನೀರ್ ತಂಪು ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>This water is cold</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಆ ಕೋಣೆ ಎಲ್ಯ ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>That room is small</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಈ ಪುಸ್ತಕ ಕುತೂಹಲಕಾರಿ ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>This book is interesting</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ನಮ್ಮ ಊರುಡು ಶಾಂತಿಯುತವಾತ್ ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Our village is peaceful</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಈ ಪೂ ಪೊರ್ಲು ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>This flower is nice</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ಆ ಸುದೆ ಗುಂಡಿ ಉಂಡು </t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>That river is deep</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>description</t>
         </is>
       </c>
     </row>

</xml_diff>